<commit_message>
Ejercicios de empresa corregidos y revisados por el profesor
</commit_message>
<xml_diff>
--- a/EMPRESA/Ejercicio 2_producción a corto plazo.xlsx
+++ b/EMPRESA/Ejercicio 2_producción a corto plazo.xlsx
@@ -620,10 +620,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.0604752970606629"/>
-          <c:y val="0.0458083166555481"/>
-          <c:w val="0.896122576610382"/>
-          <c:h val="0.865577051367578"/>
+          <c:x val="0.0604736878028804"/>
+          <c:y val="0.045752427184466"/>
+          <c:w val="0.896048051327554"/>
+          <c:h val="0.865412621359223"/>
         </c:manualLayout>
       </c:layout>
       <c:scatterChart>
@@ -1109,11 +1109,11 @@
           </c:yVal>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="63355692"/>
-        <c:axId val="75884541"/>
+        <c:axId val="96750414"/>
+        <c:axId val="99535134"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="63355692"/>
+        <c:axId val="96750414"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1146,12 +1146,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="75884541"/>
+        <c:crossAx val="99535134"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="75884541"/>
+        <c:axId val="99535134"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1193,7 +1193,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="63355692"/>
+        <c:crossAx val="96750414"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1399,7 +1399,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Beneficio Maximo 1496</c:v>
+                  <c:v>Beneficio Maximo 112 q(vespas)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1656,11 +1656,11 @@
           </c:yVal>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="70013370"/>
-        <c:axId val="67325196"/>
+        <c:axId val="21446888"/>
+        <c:axId val="11749879"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="70013370"/>
+        <c:axId val="21446888"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1693,12 +1693,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="67325196"/>
+        <c:crossAx val="11749879"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="67325196"/>
+        <c:axId val="11749879"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1740,7 +1740,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="70013370"/>
+        <c:crossAx val="21446888"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -2117,11 +2117,11 @@
           </c:yVal>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="44259349"/>
-        <c:axId val="51548811"/>
+        <c:axId val="85299217"/>
+        <c:axId val="35988033"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="44259349"/>
+        <c:axId val="85299217"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2154,12 +2154,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="51548811"/>
+        <c:crossAx val="35988033"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="51548811"/>
+        <c:axId val="35988033"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2201,7 +2201,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="44259349"/>
+        <c:crossAx val="85299217"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -2266,10 +2266,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.0614139267408426"/>
-          <c:y val="0.0645143365192265"/>
-          <c:w val="0.697524690586323"/>
-          <c:h val="0.864747721715937"/>
+          <c:x val="0.0614272809394761"/>
+          <c:y val="0.064474842012639"/>
+          <c:w val="0.69747539580659"/>
+          <c:h val="0.864650827933765"/>
         </c:manualLayout>
       </c:layout>
       <c:scatterChart>
@@ -2566,11 +2566,11 @@
           </c:marker>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="84890844"/>
-        <c:axId val="47625876"/>
+        <c:axId val="97962532"/>
+        <c:axId val="30393300"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="84890844"/>
+        <c:axId val="97962532"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2603,12 +2603,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="47625876"/>
+        <c:crossAx val="30393300"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="47625876"/>
+        <c:axId val="30393300"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2650,7 +2650,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="84890844"/>
+        <c:crossAx val="97962532"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -2724,9 +2724,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>784800</xdr:colOff>
+      <xdr:colOff>784440</xdr:colOff>
       <xdr:row>45</xdr:row>
-      <xdr:rowOff>136440</xdr:rowOff>
+      <xdr:rowOff>136080</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2735,7 +2735,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="852120" y="6171120"/>
-        <a:ext cx="5274360" cy="2966400"/>
+        <a:ext cx="5274000" cy="2966040"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2754,9 +2754,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>18</xdr:col>
-      <xdr:colOff>818640</xdr:colOff>
+      <xdr:colOff>818280</xdr:colOff>
       <xdr:row>45</xdr:row>
-      <xdr:rowOff>87120</xdr:rowOff>
+      <xdr:rowOff>86760</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2765,7 +2765,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="11087640" y="5850720"/>
-        <a:ext cx="5756040" cy="3237480"/>
+        <a:ext cx="5755680" cy="3237120"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2784,9 +2784,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>453240</xdr:colOff>
+      <xdr:colOff>452880</xdr:colOff>
       <xdr:row>16</xdr:row>
-      <xdr:rowOff>74160</xdr:rowOff>
+      <xdr:rowOff>73800</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2795,7 +2795,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="926640" y="36000"/>
-        <a:ext cx="5758560" cy="3238560"/>
+        <a:ext cx="5758200" cy="3238200"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2814,9 +2814,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>18</xdr:col>
-      <xdr:colOff>258120</xdr:colOff>
+      <xdr:colOff>257760</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>180000</xdr:rowOff>
+      <xdr:rowOff>179640</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2825,7 +2825,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="8711280" y="480240"/>
-        <a:ext cx="7571880" cy="4500360"/>
+        <a:ext cx="7571520" cy="4500000"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -4198,27 +4198,27 @@
       <c r="B26" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C26" s="0" t="n">
+      <c r="C26" s="7" t="n">
         <f aca="false">MAX('Tabla de producción'!O5:O15)</f>
         <v>1496</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E28" s="0" t="s">
+      <c r="E28" s="7" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="7" t="str">
-        <f aca="false">CONCATENATE(B26," ",C26)</f>
-        <v>Beneficio Maximo 1496</v>
-      </c>
-      <c r="E29" s="0" t="s">
+        <f aca="false">CONCATENATE(B26," ",'Tabla de producción'!J21," ",Datos!C7)</f>
+        <v>Beneficio Maximo 112 q(vespas)</v>
+      </c>
+      <c r="E29" s="7" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E31" s="0" t="str">
+      <c r="E31" s="7" t="str">
         <f aca="false">CONCATENATE(E28,B19,E29)</f>
         <v>Ley de los redimientos decrecientes cuando hay 3 trabajadores</v>
       </c>

</xml_diff>